<commit_message>
Raise BQU3875's capacity to 23.0T (real-world correction)
MUATAN's "LORRY NAIK (10%)" had BQU3875 at 22.0T, still 0.56T short of
the 9-DO Kuantan route total (22.5592T), so even after syncing
master_lorry.xlsx to MUATAN it still spilled one DO onto a second
lorry. Confirmed with the user this was MUATAN's figure being
conservative, not a real safety limit — BQU3875 actually handles up to
23T. Updated both LORRY DAILY PLANNING.xlsx's MUATAN sheet and
master_lorry.xlsx to 23.0T so they stay in sync.

Verified: all 9 Kuantan DOs (22.559T) now consolidate onto BQU3875
alone (98.1% utilized), freeing BQY7823 entirely. Diffed the resaved
workbook cell-by-cell against the original — all 12 sheets intact,
only the intended MUATAN cell changed.
</commit_message>
<xml_diff>
--- a/data/master_lorry.xlsx
+++ b/data/master_lorry.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
-        <v>22000</v>
+        <v>23000</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>

</xml_diff>